<commit_message>
Added column2 via test branch
</commit_message>
<xml_diff>
--- a/123.xlsx
+++ b/123.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyPythonProjects\yandexDLE\test_git\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D8C5393-4F2B-4A98-AD72-54B9964F552D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07CCC5ED-84CE-4B7C-AA82-A5A06BCFE1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4230" yWindow="2535" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,9 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t>column1</t>
+  </si>
+  <si>
+    <t>column2</t>
   </si>
 </sst>
 </file>
@@ -345,40 +348,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>13</v>
       </c>

</xml_diff>